<commit_message>
GDTC 1–5: đồng bộ theo app bản 170 — cột 7 chép từ giáo án, lớp 1 số tiết cả bài, lớp 4 bỏ tiền tố dòng 1 (website + web-chung sinh lại)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/docs/lop1/Giao duc the chat - Lop 1.xlsx
+++ b/assets/docs/lop1/Giao duc the chat - Lop 1.xlsx
@@ -547,7 +547,7 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>3 tiết</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
@@ -582,7 +582,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>3 tiết</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -616,7 +616,7 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>3 tiết</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
@@ -650,7 +650,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>4 tiết</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -685,7 +685,7 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>4 tiết</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -719,7 +719,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>4 tiết</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -754,7 +754,7 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>4 tiết</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
@@ -788,7 +788,7 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>4 tiết</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
@@ -823,7 +823,7 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>4 tiết</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
@@ -857,7 +857,7 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>4 tiết</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
@@ -892,7 +892,7 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>4 tiết</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
@@ -926,7 +926,7 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>3 tiết</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
@@ -961,7 +961,7 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>3 tiết</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
@@ -995,7 +995,7 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>3 tiết</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
@@ -1029,7 +1029,7 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>2 tiết</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
@@ -1063,7 +1063,7 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>2 tiết</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
@@ -1093,7 +1093,7 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>3 tiết</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
@@ -1127,7 +1127,7 @@
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>3 tiết</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
@@ -1157,7 +1157,7 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>3 tiết</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
@@ -1191,7 +1191,7 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>2 tiết</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
@@ -1225,7 +1225,7 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>2 tiết</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
@@ -1289,7 +1289,7 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>3 tiết</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
@@ -1324,7 +1324,7 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>3 tiết</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
@@ -1358,7 +1358,7 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>3 tiết</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
@@ -1392,7 +1392,7 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>4 tiết</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>4 tiết</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
@@ -1461,7 +1461,7 @@
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>4 tiết</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
@@ -1496,7 +1496,7 @@
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>4 tiết</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
@@ -1530,7 +1530,7 @@
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>5 tiết</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
@@ -1565,7 +1565,7 @@
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>5 tiết</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
@@ -1599,7 +1599,7 @@
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>5 tiết</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
@@ -1634,7 +1634,7 @@
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>5 tiết</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
@@ -1668,7 +1668,7 @@
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>5 tiết</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
@@ -1766,7 +1766,7 @@
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>6 tiết</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
@@ -1801,7 +1801,7 @@
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>6 tiết</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
@@ -1835,7 +1835,7 @@
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>6 tiết</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
@@ -1870,7 +1870,7 @@
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>6 tiết</t>
         </is>
       </c>
       <c r="G43" s="4" t="inlineStr">
@@ -1904,7 +1904,7 @@
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>6 tiết</t>
         </is>
       </c>
       <c r="G44" s="4" t="inlineStr">
@@ -1939,7 +1939,7 @@
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>6 tiết</t>
         </is>
       </c>
       <c r="G45" s="4" t="inlineStr">
@@ -1973,7 +1973,7 @@
       </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>6 tiết</t>
         </is>
       </c>
       <c r="G46" s="4" t="inlineStr">
@@ -2008,7 +2008,7 @@
       </c>
       <c r="F47" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>6 tiết</t>
         </is>
       </c>
       <c r="G47" s="4" t="inlineStr">
@@ -2042,7 +2042,7 @@
       </c>
       <c r="F48" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>6 tiết</t>
         </is>
       </c>
       <c r="G48" s="4" t="inlineStr">
@@ -2077,7 +2077,7 @@
       </c>
       <c r="F49" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>6 tiết</t>
         </is>
       </c>
       <c r="G49" s="4" t="inlineStr">
@@ -2111,7 +2111,7 @@
       </c>
       <c r="F50" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>6 tiết</t>
         </is>
       </c>
       <c r="G50" s="4" t="inlineStr">
@@ -2146,7 +2146,7 @@
       </c>
       <c r="F51" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>6 tiết</t>
         </is>
       </c>
       <c r="G51" s="4" t="inlineStr">
@@ -2180,7 +2180,7 @@
       </c>
       <c r="F52" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>4 tiết</t>
         </is>
       </c>
       <c r="G52" s="4" t="inlineStr">
@@ -2214,7 +2214,7 @@
       </c>
       <c r="F53" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>4 tiết</t>
         </is>
       </c>
       <c r="G53" s="4" t="inlineStr">
@@ -2244,7 +2244,7 @@
       </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>4 tiết</t>
         </is>
       </c>
       <c r="G54" s="4" t="inlineStr">
@@ -2274,7 +2274,7 @@
       </c>
       <c r="F55" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>4 tiết</t>
         </is>
       </c>
       <c r="G55" s="4" t="inlineStr">
@@ -2308,7 +2308,7 @@
       </c>
       <c r="F56" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>4 tiết</t>
         </is>
       </c>
       <c r="G56" s="4" t="inlineStr">
@@ -2342,7 +2342,7 @@
       </c>
       <c r="F57" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>4 tiết</t>
         </is>
       </c>
       <c r="G57" s="4" t="inlineStr">
@@ -2372,7 +2372,7 @@
       </c>
       <c r="F58" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>4 tiết</t>
         </is>
       </c>
       <c r="G58" s="4" t="inlineStr">
@@ -2402,7 +2402,7 @@
       </c>
       <c r="F59" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>4 tiết</t>
         </is>
       </c>
       <c r="G59" s="4" t="inlineStr">
@@ -2470,7 +2470,7 @@
       </c>
       <c r="F61" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>5 tiết</t>
         </is>
       </c>
       <c r="G61" s="4" t="inlineStr">
@@ -2504,7 +2504,7 @@
       </c>
       <c r="F62" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>5 tiết</t>
         </is>
       </c>
       <c r="G62" s="4" t="inlineStr">
@@ -2534,7 +2534,7 @@
       </c>
       <c r="F63" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>5 tiết</t>
         </is>
       </c>
       <c r="G63" s="4" t="inlineStr">
@@ -2564,7 +2564,7 @@
       </c>
       <c r="F64" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>5 tiết</t>
         </is>
       </c>
       <c r="G64" s="4" t="inlineStr">
@@ -2598,7 +2598,7 @@
       </c>
       <c r="F65" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>5 tiết</t>
         </is>
       </c>
       <c r="G65" s="4" t="inlineStr">
@@ -2628,7 +2628,7 @@
       </c>
       <c r="F66" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>5 tiết</t>
         </is>
       </c>
       <c r="G66" s="4" t="inlineStr">
@@ -2662,7 +2662,7 @@
       </c>
       <c r="F67" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>5 tiết</t>
         </is>
       </c>
       <c r="G67" s="4" t="inlineStr">
@@ -2692,7 +2692,7 @@
       </c>
       <c r="F68" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>5 tiết</t>
         </is>
       </c>
       <c r="G68" s="4" t="inlineStr">
@@ -2722,7 +2722,7 @@
       </c>
       <c r="F69" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>5 tiết</t>
         </is>
       </c>
       <c r="G69" s="4" t="inlineStr">
@@ -2756,7 +2756,7 @@
       </c>
       <c r="F70" s="4" t="inlineStr">
         <is>
-          <t>1 tiết</t>
+          <t>5 tiết</t>
         </is>
       </c>
       <c r="G70" s="4" t="inlineStr">

</xml_diff>